<commit_message>
Minor variable name adjustment
</commit_message>
<xml_diff>
--- a/dictionary/variable_dictionary.xlsx
+++ b/dictionary/variable_dictionary.xlsx
@@ -492,13 +492,13 @@
     <t xml:space="preserve">Deflator do rendimento habitual (IBGE, base trimestral)</t>
   </si>
   <si>
-    <t xml:space="preserve">Habitual income deflator (IBGE, quarterly base)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Real number between 0 and 1. Multiply by VD4019 to get real income.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rendimento_habitual_real</t>
+    <t xml:space="preserve">Habitual earnings deflator (IBGE, quarterly base)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Real number between 0 and 1. Multiply by VD4019 to get real earnings.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">earnings_habitual_real</t>
   </si>
   <si>
     <t xml:space="preserve">Rendimento mensal habitual real de todos os trabalhos (VD4019 × Habitual, em R$)</t>
@@ -507,7 +507,7 @@
     <t xml:space="preserve">Real habitual monthly earnings from all jobs (VD4019 × Habitual, in R$)</t>
   </si>
   <si>
-    <t xml:space="preserve">Positive real or NA. Main income variable for analysis.</t>
+    <t xml:space="preserve">Positive real or NA. Main earnings variable for analysis.</t>
   </si>
   <si>
     <t xml:space="preserve">VD4031</t>

</xml_diff>